<commit_message>
inherit implemented for campaign, sampling_log, observation_log
</commit_message>
<xml_diff>
--- a/lucas/import_data/dataset_meta/excel/campaign.xlsx
+++ b/lucas/import_data/dataset_meta/excel/campaign.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
   <si>
     <t xml:space="preserve">dataset_id__dataset_name</t>
   </si>
@@ -109,6 +109,12 @@
     <t xml:space="preserve">LUCAS 2009</t>
   </si>
   <si>
+    <t xml:space="preserve">inherit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://esdac.jrc.ec.europa.eu/content/lucas-2009-topsoil-data</t>
+  </si>
+  <si>
     <t xml:space="preserve">LUCAS</t>
   </si>
   <si>
@@ -134,6 +140,9 @@
   </si>
   <si>
     <t xml:space="preserve">LUCAS 2015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://esdac.jrc.ec.europa.eu/content/lucas2015-topsoil-data</t>
   </si>
   <si>
     <t xml:space="preserve">foss xds rca,lucas-wetlab-2015</t>
@@ -146,7 +155,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -167,6 +176,13 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -211,7 +227,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -225,6 +241,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -360,6 +380,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="24.04"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="23.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="23.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="20.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="20.93"/>
@@ -458,38 +479,47 @@
       <c r="C2" s="1" t="s">
         <v>28</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="F2" s="1" t="n">
         <v>20090501</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>20091031</v>
       </c>
+      <c r="H2" s="1" t="s">
+        <v>30</v>
+      </c>
       <c r="J2" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="N2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="T2" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="U2" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="V2" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="W2" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="X2" s="1" t="n">
         <v>1000</v>
       </c>
       <c r="Y2" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Z2" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -497,10 +527,16 @@
         <v>26</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>20150501</v>
@@ -508,35 +544,41 @@
       <c r="G3" s="1" t="n">
         <v>20151031</v>
       </c>
+      <c r="H3" s="4" t="s">
+        <v>40</v>
+      </c>
       <c r="J3" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="N3" s="1" t="n">
         <v>1</v>
       </c>
       <c r="T3" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="W3" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="X3" s="1" t="n">
         <v>1000</v>
       </c>
       <c r="Y3" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H3" r:id="rId1" display="https://esdac.jrc.ec.europa.eu/content/lucas2015-topsoil-data"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.025" bottom="1.025" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>